<commit_message>
Sin referencias al Ministerio: plantillas de Excel limpias (pie, institucion, enlaces externos), institucion sin valor por defecto; pantalla Acerca de con licencias, plantilla propia de Excel e informe de errores; compilacion de produccion con R8 probada, paquete de mapas aparte para Play, Compose alineado entre depuracion y publicacion; pruebas de respaldo y de carga; documentos legales
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/src/main/assets/ficha_familiar.xlsx
+++ b/app/src/main/assets/ficha_familiar.xlsx
@@ -1,12 +1,12 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x15 xr xr6 xr10 xr2" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2"><fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/><workbookPr/><mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006"><mc:Choice Requires="x15"><x15ac:absPath url="C:\Users\MSI\Desktop\" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac"/></mc:Choice></mc:AlternateContent><xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E11F210-10C0-4C64-9F24-CFCBC5AC62D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/><bookViews><workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/></bookViews><sheets><sheet name="1" sheetId="1" r:id="rId1"/><sheet name="2" sheetId="2" r:id="rId2"/><sheet name="3" sheetId="3" r:id="rId3"/><sheet name="4" sheetId="4" r:id="rId4"/></sheets><externalReferences><externalReference r:id="rId5"/><externalReference r:id="rId6"/></externalReferences><definedNames><definedName name="_xlnm.Print_Area" localSheetId="0">'1'!$A$1:$CZ$47</definedName><definedName name="_xlnm.Print_Area" localSheetId="1">'2'!$A$1:$CV$49</definedName><definedName name="_xlnm.Print_Area" localSheetId="2">'3'!$B$1:$CW$28</definedName><definedName name="_xlnm.Print_Area" localSheetId="3">'4'!$B$1:$CS$50</definedName><definedName name="TOTAL" localSheetId="1">[2]PLANPROSA!IW65537</definedName><definedName name="TOTAL">[1]PLANPROSA!IW65537</definedName></definedNames><calcPr calcId="191029" iterateDelta="1E-4"/><extLst><ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures"><xcalcf:calcFeatures><xcalcf:feature name="microsoft.com:RD"/><xcalcf:feature name="microsoft.com:Single"/><xcalcf:feature name="microsoft.com:FV"/><xcalcf:feature name="microsoft.com:CNMTM"/><xcalcf:feature name="microsoft.com:LET_WF"/><xcalcf:feature name="microsoft.com:LAMBDA_WF"/><xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/></xcalcf:calcFeatures></ext><ext uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}"><ns2:extCalcPr stringRefSyntax="CalcA1"/></ext></extLst></workbook>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x15 xr xr6 xr10 xr2" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2"><fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/><workbookPr/><mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006"><mc:Choice Requires="x15"><x15ac:absPath url="C:\Users\MSI\Desktop\" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac"/></mc:Choice></mc:AlternateContent><xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E11F210-10C0-4C64-9F24-CFCBC5AC62D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/><bookViews><workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/></bookViews><sheets><sheet name="1" sheetId="1" r:id="rId1"/><sheet name="2" sheetId="2" r:id="rId2"/><sheet name="3" sheetId="3" r:id="rId3"/><sheet name="4" sheetId="4" r:id="rId4"/></sheets><definedNames><definedName name="_xlnm.Print_Area" localSheetId="0">'1'!$A$1:$CZ$47</definedName><definedName name="_xlnm.Print_Area" localSheetId="1">'2'!$A$1:$CV$49</definedName><definedName name="_xlnm.Print_Area" localSheetId="2">'3'!$B$1:$CW$28</definedName><definedName name="_xlnm.Print_Area" localSheetId="3">'4'!$B$1:$CS$50</definedName></definedNames><calcPr calcId="191029" iterateDelta="1E-4"/><extLst><ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures"><xcalcf:calcFeatures><xcalcf:feature name="microsoft.com:RD"/><xcalcf:feature name="microsoft.com:Single"/><xcalcf:feature name="microsoft.com:FV"/><xcalcf:feature name="microsoft.com:CNMTM"/><xcalcf:feature name="microsoft.com:LET_WF"/><xcalcf:feature name="microsoft.com:LAMBDA_WF"/><xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/></xcalcf:calcFeatures></ext><ext uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}"><ns2:extCalcPr stringRefSyntax="CalcA1"/></ext></extLst></workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="170">
   <si>
-    <t>INSTITUCIÓN DEL SISTEMA</t>
+    <t>INSTITUCIÓN</t>
   </si>
   <si>
     <t>UNIDAD OPERATIVA</t>
@@ -287,7 +287,7 @@
     <t>FICHA FAMILIAR - ANAMNESIS</t>
   </si>
   <si>
-    <t>SNS-MSP / HCU-anexo 1 / 2008 (hoja 1)</t>
+    <t>Ficha familiar (hoja 1)</t>
   </si>
   <si>
     <t>CALIFICACION DEL RIESGO FAMILIAR</t>
@@ -444,7 +444,7 @@
     <t>RESPONSABLE DE LA CALIFICACION</t>
   </si>
   <si>
-    <t>SNS-MSP / HCU-anexo 1 / 2008 (hoja 2)</t>
+    <t>Ficha familiar (hoja 2)</t>
   </si>
   <si>
     <t>FICHA FAMILIAR - RIESGOS</t>
@@ -524,7 +524,7 @@
     <t>RESPONSABLE</t>
   </si>
   <si>
-    <t>SNS-MSP / HCU-anexo 1 / 2008 (hoja 3)</t>
+    <t>Ficha familiar (hoja 3)</t>
   </si>
   <si>
     <t>FICHA FAMILIAR - EVOLUCION</t>
@@ -615,7 +615,7 @@
     <t>LUGAR O PERSONA A LA QUE ACUDEN PARA TRATAMIENTO</t>
   </si>
   <si>
-    <t>SNS-MSP / HCU-anexo 1 / 2008 (hoja 4)</t>
+    <t>Ficha familiar (hoja 4)</t>
   </si>
   <si>
     <t>FICHA FAMILIAR - FAMILIOGRAMA Y CONTAMINACION</t>
@@ -6887,174 +6887,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:relativeUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="C-PPS"/>
-      <sheetName val="C-Xp"/>
-      <sheetName val="C-Yp"/>
-      <sheetName val="C-Zp"/>
-      <sheetName val="C-1P"/>
-      <sheetName val="C-2p"/>
-      <sheetName val="C-3p"/>
-      <sheetName val="C-4p"/>
-      <sheetName val="C-5p"/>
-      <sheetName val="C-6p"/>
-      <sheetName val="C-7p"/>
-      <sheetName val="C-8p"/>
-      <sheetName val="C-9p"/>
-      <sheetName val="C-10p"/>
-      <sheetName val="C- 11p"/>
-      <sheetName val="C-12p"/>
-      <sheetName val="F-1p"/>
-      <sheetName val="F- 2p"/>
-      <sheetName val="F- 3p"/>
-      <sheetName val="F- 4p"/>
-      <sheetName val="F- 5p"/>
-      <sheetName val="F- 6p"/>
-      <sheetName val="F- 7p"/>
-      <sheetName val="F- 8p"/>
-      <sheetName val="F- 9p"/>
-      <sheetName val="F-10p"/>
-      <sheetName val="F-11p"/>
-      <sheetName val="F-Ap"/>
-      <sheetName val="F-Bp"/>
-      <sheetName val="F- Cp"/>
-      <sheetName val="F- Dp"/>
-      <sheetName val="F- Ep"/>
-      <sheetName val="F- Fp"/>
-      <sheetName val="F-Gp"/>
-      <sheetName val="PLANPROSA"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:relativeUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="C-PPS"/>
-      <sheetName val="C-Xp"/>
-      <sheetName val="C-Yp"/>
-      <sheetName val="C-Zp"/>
-      <sheetName val="C-1P"/>
-      <sheetName val="C-2p"/>
-      <sheetName val="C-3p"/>
-      <sheetName val="C-4p"/>
-      <sheetName val="C-5p"/>
-      <sheetName val="C-6p"/>
-      <sheetName val="C-7p"/>
-      <sheetName val="C-8p"/>
-      <sheetName val="C-9p"/>
-      <sheetName val="C-10p"/>
-      <sheetName val="C- 11p"/>
-      <sheetName val="C-12p"/>
-      <sheetName val="F-1p"/>
-      <sheetName val="F- 2p"/>
-      <sheetName val="F- 3p"/>
-      <sheetName val="F- 4p"/>
-      <sheetName val="F- 5p"/>
-      <sheetName val="F- 6p"/>
-      <sheetName val="F- 7p"/>
-      <sheetName val="F- 8p"/>
-      <sheetName val="F- 9p"/>
-      <sheetName val="F-10p"/>
-      <sheetName val="F-11p"/>
-      <sheetName val="F-Ap"/>
-      <sheetName val="F-Bp"/>
-      <sheetName val="F- Cp"/>
-      <sheetName val="F- Dp"/>
-      <sheetName val="F- Ep"/>
-      <sheetName val="F- Fp"/>
-      <sheetName val="F-Gp"/>
-      <sheetName val="PLANPROSA"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>